<commit_message>
Add a Default agents sort setting, alongside Default view
Same pattern as Default view: a dropdown in the workbook's SETTINGS section
(cell B5, 'Legend & how to use'), read by build_data.py and mapped to the
internal sort key the Agents by phase view's own Sort buttons already use
(A to Z / Most advanced / Class / Stage / Entry type). Blank keeps A to Z,
same as before; a value outside the five options stops the build with a
row-style message, same as every other checked field.

This fills the gap in the previous default_view work: default_timeline_order
only takes effect when the timeline is what opens first, so setting Default
view to Agents by phase (as this workbook now does) left no way to control
what order THAT view opened in. Tested: blank keeps A to Z, 'Most advanced'
changes it, a typo is rejected before the build writes anything, and restored
to blank before committing so the live site's behaviour is unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hiv_curation.xlsx
+++ b/hiv_curation.xlsx
@@ -5121,7 +5121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="34" min="1" max="1"/>
@@ -5168,335 +5168,358 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="34"/>
+    <row r="5" ht="15" customHeight="1" s="34">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>Default agents sort</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>A to Z</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="39" customHeight="1" s="34">
-      <c r="A6" s="11" t="n"/>
-      <c r="B6" s="12" t="n"/>
-    </row>
-    <row r="7" ht="23.75" customHeight="1" s="34">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>The starting sort for the Agents by phase view, matching its own Sort buttons. Leave blank to keep A to Z. Only matters if that view is what Default view opens on, or once someone visits it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="23.75" customHeight="1" s="34"/>
+    <row r="8" ht="15" customHeight="1" s="34">
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="34">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>HOW IT WORKS</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="34">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>1. Edit the Entries tab</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>One row per product. Change any white cell. Add or delete whole rows freely; order does not matter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="34">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>2. Save the file</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Keep it as .xlsx.</t>
-        </is>
-      </c>
+      <c r="B9" s="14" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="34">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>3. Run the build step</t>
+          <t>1. Edit the Entries tab</t>
         </is>
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>In a terminal:  python build_data.py hiv_curation.xlsx  → writes hiv_dashboard_data.json, which the dashboard reads.</t>
+          <t>One row per product. Change any white cell. Add or delete whole rows freely; order does not matter.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="34">
       <c r="A11" s="11" t="inlineStr">
         <is>
+          <t>2. Save the file</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Keep it as .xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="34">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>3. Run the build step</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>In a terminal:  python build_data.py hiv_curation.xlsx  → writes hiv_dashboard_data.json, which the dashboard reads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="23.75" customHeight="1" s="34">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
           <t>4. Refresh the dashboard</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>The new data appears. The build step prints a check report and refuses to write if something essential is missing.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="34">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="12" t="n"/>
-    </row>
-    <row r="13" ht="23.75" customHeight="1" s="34">
-      <c r="A13" s="13" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="34">
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="12" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="34">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>COLUMNS</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n"/>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="34">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>Leave as is. Leave blank for a new row and the build step assigns one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="34">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>band</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>formulations = a discrete long-acting product. compounds = an underlying molecule in LA development.</t>
-        </is>
-      </c>
+      <c r="B15" s="14" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="34">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Product or molecule name, shown on the dashboard.</t>
+          <t>Leave as is. Leave blank for a new row and the build step assigns one.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="34">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>indication</t>
+          <t>band</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Treatment, Prevention, or Both. Drives which selection the row appears under. "Both" shows it once, tagged for both.</t>
+          <t>formulations = a discrete long-acting product. compounds = an underlying molecule in LA development.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="23.75" customHeight="1" s="34">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>stage</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>Approved / Late-stage / Early-stage / Not stated. Sets the row colour and grouping.</t>
+          <t>Product or molecule name, shown on the dashboard.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="23.75" customHeight="1" s="34">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>highest_phase</t>
+          <t>indication</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>Highest clinical phase on record. Optional, shown in the tooltip.</t>
+          <t>Treatment, Prevention, or Both. Drives which selection the row appears under. "Both" shows it once, tagged for both.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="23.75" customHeight="1" s="34">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>developers</t>
+          <t>stage</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>One or more, separated by a semicolon ( ; ).</t>
+          <t>Approved / Late-stage / Early-stage / Not stated. Sets the row colour and grouping.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="34">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>drug_class</t>
+          <t>highest_phase</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>Optional, shown in the tooltip.</t>
+          <t>Highest clinical phase on record. Optional, shown in the tooltip.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="34">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>ROUTE columns</t>
+          <t>developers</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>Mark x under every route that applies. PO oral, SC subcutaneous, IM intramuscular, IV intravenous, VR vaginal ring, TD transdermal.</t>
+          <t>One or more, separated by a semicolon ( ; ).</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="34">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>INTERVAL columns</t>
+          <t>drug_class</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Mark x under every dosing interval studied. 1W weekly, 2W 2-weekly, 1M monthly, 2M, 3M, 4M, 6M, 12M yearly. Leave all blank if unknown; the row then sits in the "not stated" lane. Do not enter daily or single-dose.</t>
+          <t>Optional, shown in the tooltip.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="34">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>frequency_source</t>
+          <t>ROUTE columns</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>LAPaL record = confirmed. "derived from trials" = filled from a linked trial and shown with a dagger until you confirm. Change to "manually confirmed" once checked.</t>
+          <t>Mark x under every route that applies. PO oral, SC subcutaneous, IM intramuscular, IV intravenous, VR vaginal ring, TD transdermal.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="34">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>flag_no_trials</t>
+          <t>INTERVAL columns</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Mark x if no clinical trials are linked in LAPaL. Surfaced in the data-quality panel.</t>
+          <t>Mark x under every dosing interval studied. 1W weekly, 2W 2-weekly, 1M monthly, 2M, 3M, 4M, 6M, 12M yearly. Leave all blank if unknown; the row then sits in the "not stated" lane. Do not enter daily or single-dose.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="34">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>flag_no_reg_rows</t>
+          <t>frequency_source</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Mark x if approved but missing structured regulatory rows. Surfaced in the data-quality panel.</t>
+          <t>LAPaL record = confirmed. "derived from trials" = filled from a linked trial and shown with a dagger until you confirm. Change to "manually confirmed" once checked.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="23.75" customHeight="1" s="34">
       <c r="A27" s="11" t="inlineStr">
         <is>
+          <t>flag_no_trials</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Mark x if no clinical trials are linked in LAPaL. Surfaced in the data-quality panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="34">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>flag_no_reg_rows</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Mark x if approved but missing structured regulatory rows. Surfaced in the data-quality panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="34">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
           <t>curator_notes</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Free text for you. Not shown on the dashboard.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="34">
-      <c r="A28" s="11" t="n"/>
-      <c r="B28" s="12" t="n"/>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="34">
-      <c r="A29" s="13" t="inlineStr">
+    <row r="30" ht="15" customHeight="1" s="34">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="12" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="34">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>AUTOMATIC FLAGS</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B31" s="14" t="inlineStr">
         <is>
           <t>The build step computes these; you do not enter them:</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="34">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>missing_frequency</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>set when no interval x is marked.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="34">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>conventional_approval_only</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>set when stage is Approved, no interval is marked, and the only route is oral (an approved conventional drug shown as an API in LA development).</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="n"/>
-      <c r="B32" s="12" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="11" t="n"/>
+      <c r="B34" s="12" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>RULES THE BUILD STEP CHECKS</t>
         </is>
       </c>
-      <c r="B33" s="16" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="B35" s="16" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>every row needs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>a band, a name, an indication and a stage. Missing any of these stops the build with a clear message.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>controlled values</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>band, stage, indication and interval codes must match the lists above. Typos are reported by row.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" s="34"/>
-    <row r="44" ht="16" customHeight="1" s="34">
-      <c r="A44" s="26" t="inlineStr">
+    <row r="44" ht="16" customHeight="1" s="34"/>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
         <is>
           <t>Example: to add a product, copy a row, change name, set band/indication/stage, mark x under each route and interval, leave id blank. Then run build_data.py.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Dosing timeline,Agents by phase,Class and phase,Counts"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A to Z,Most advanced,Class,Stage,Entry type"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>